<commit_message>
DSV.CO PP&E, STD and excel
</commit_message>
<xml_diff>
--- a/data/cox_xlsx/DSV.CO.xlsx
+++ b/data/cox_xlsx/DSV.CO.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="886" uniqueCount="459">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="886" uniqueCount="461">
   <si>
     <t>Company Fundamentals - Income Statement</t>
   </si>
@@ -855,6 +855,9 @@
     <t>Lease liabilities</t>
   </si>
   <si>
+    <t>Borrowings (not use)</t>
+  </si>
+  <si>
     <t>Borrowings</t>
   </si>
   <si>
@@ -889,6 +892,9 @@
   </si>
   <si>
     <t>Assets Held for Sale</t>
+  </si>
+  <si>
+    <t>Borrowings 2</t>
   </si>
   <si>
     <t>Total current liabilities</t>
@@ -13134,8 +13140,14 @@
       <c r="N61" s="16">
         <v>4341.06</v>
       </c>
-      <c r="O61" s="15"/>
-      <c r="P61" s="15"/>
+      <c r="O61" s="19">
+        <f t="shared" ref="O61:P61" si="1">O62+O65+O68</f>
+        <v>4194.5</v>
+      </c>
+      <c r="P61" s="19">
+        <f t="shared" si="1"/>
+        <v>4686.16</v>
+      </c>
       <c r="Q61" s="16">
         <v>4998.0</v>
       </c>
@@ -14436,7 +14448,7 @@
       <c r="W86" s="15"/>
     </row>
     <row r="87" ht="15.0" customHeight="1">
-      <c r="A87" s="14" t="s">
+      <c r="A87" s="24" t="s">
         <v>278</v>
       </c>
       <c r="B87" s="15"/>
@@ -14466,7 +14478,7 @@
     </row>
     <row r="88" ht="15.0" customHeight="1">
       <c r="A88" s="14" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B88" s="15"/>
       <c r="C88" s="15"/>
@@ -14505,7 +14517,7 @@
     </row>
     <row r="89" ht="15.0" customHeight="1">
       <c r="A89" s="14" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B89" s="15">
         <v>15905.96</v>
@@ -14562,7 +14574,7 @@
     </row>
     <row r="90" ht="15.0" customHeight="1">
       <c r="A90" s="14" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B90" s="15">
         <v>37163.47</v>
@@ -14633,7 +14645,7 @@
     </row>
     <row r="91" ht="15.0" customHeight="1">
       <c r="A91" s="14" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B91" s="15">
         <v>20131.2</v>
@@ -14672,7 +14684,7 @@
     </row>
     <row r="92" ht="15.0" customHeight="1">
       <c r="A92" s="14" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B92" s="15">
         <v>10264.92</v>
@@ -14743,7 +14755,7 @@
     </row>
     <row r="93" ht="15.0" customHeight="1">
       <c r="A93" s="14" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B93" s="15"/>
       <c r="C93" s="15"/>
@@ -14774,7 +14786,7 @@
     </row>
     <row r="94" ht="15.0" customHeight="1">
       <c r="A94" s="14" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B94" s="15"/>
       <c r="C94" s="15"/>
@@ -14805,7 +14817,7 @@
     </row>
     <row r="95" ht="15.0" customHeight="1">
       <c r="A95" s="14" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B95" s="15"/>
       <c r="C95" s="15"/>
@@ -14836,7 +14848,7 @@
     </row>
     <row r="96" ht="15.0" customHeight="1">
       <c r="A96" s="14" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B96" s="15">
         <v>30237.94</v>
@@ -14901,7 +14913,7 @@
     </row>
     <row r="97" ht="15.0" customHeight="1">
       <c r="A97" s="14" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B97" s="16">
         <v>5645.79</v>
@@ -14972,7 +14984,7 @@
     </row>
     <row r="98" ht="15.0" customHeight="1">
       <c r="A98" s="14" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B98" s="15"/>
       <c r="C98" s="15"/>
@@ -15009,7 +15021,7 @@
     </row>
     <row r="99" ht="15.0" customHeight="1">
       <c r="A99" s="14" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B99" s="15"/>
       <c r="C99" s="15"/>
@@ -15045,7 +15057,7 @@
       <c r="W99" s="15"/>
     </row>
     <row r="100" ht="15.0" customHeight="1">
-      <c r="A100" s="14" t="s">
+      <c r="A100" s="24" t="s">
         <v>278</v>
       </c>
       <c r="B100" s="15"/>
@@ -15108,8 +15120,8 @@
       </c>
     </row>
     <row r="101" ht="15.0" customHeight="1">
-      <c r="A101" s="14" t="s">
-        <v>278</v>
+      <c r="A101" s="24" t="s">
+        <v>291</v>
       </c>
       <c r="B101" s="15"/>
       <c r="C101" s="15"/>
@@ -15136,21 +15148,43 @@
       <c r="L101" s="21">
         <v>11.58</v>
       </c>
-      <c r="M101" s="15"/>
-      <c r="N101" s="15"/>
-      <c r="O101" s="15"/>
-      <c r="P101" s="15"/>
-      <c r="Q101" s="15"/>
-      <c r="R101" s="15"/>
-      <c r="S101" s="15"/>
-      <c r="T101" s="15"/>
-      <c r="U101" s="15"/>
-      <c r="V101" s="15"/>
-      <c r="W101" s="15"/>
+      <c r="M101" s="20">
+        <v>715.06</v>
+      </c>
+      <c r="N101" s="20">
+        <v>659.6</v>
+      </c>
+      <c r="O101" s="20">
+        <v>908.59</v>
+      </c>
+      <c r="P101" s="20">
+        <v>896.02</v>
+      </c>
+      <c r="Q101" s="20">
+        <v>619.79</v>
+      </c>
+      <c r="R101" s="20">
+        <v>691.19</v>
+      </c>
+      <c r="S101" s="20">
+        <v>3878.87</v>
+      </c>
+      <c r="T101" s="20">
+        <v>642.63</v>
+      </c>
+      <c r="U101" s="20">
+        <v>704.11</v>
+      </c>
+      <c r="V101" s="20">
+        <v>751.74</v>
+      </c>
+      <c r="W101" s="20">
+        <v>1079.48</v>
+      </c>
     </row>
     <row r="102" ht="15.0" customHeight="1">
       <c r="A102" s="14" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B102" s="15"/>
       <c r="C102" s="15"/>
@@ -15191,7 +15225,7 @@
     </row>
     <row r="103" ht="15.0" customHeight="1">
       <c r="A103" s="17" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B103" s="18">
         <v>130178.94</v>
@@ -15320,7 +15354,7 @@
       <c r="W104" s="15"/>
     </row>
     <row r="105" ht="15.0" customHeight="1">
-      <c r="A105" s="14" t="s">
+      <c r="A105" s="24" t="s">
         <v>278</v>
       </c>
       <c r="B105" s="15">
@@ -15380,7 +15414,7 @@
     </row>
     <row r="106" ht="15.0" customHeight="1">
       <c r="A106" s="14" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B106" s="16">
         <v>3318.82</v>
@@ -15451,7 +15485,7 @@
     </row>
     <row r="107" ht="15.0" customHeight="1">
       <c r="A107" s="14" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B107" s="16">
         <v>9377.48</v>
@@ -15522,7 +15556,7 @@
     </row>
     <row r="108" ht="15.0" customHeight="1">
       <c r="A108" s="14" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B108" s="16">
         <v>1178.51</v>
@@ -15577,7 +15611,7 @@
     </row>
     <row r="109" ht="15.0" customHeight="1">
       <c r="A109" s="14" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B109" s="16">
         <v>2084.94</v>
@@ -15632,7 +15666,7 @@
     </row>
     <row r="110" ht="15.0" customHeight="1">
       <c r="A110" s="14" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B110" s="16">
         <v>6114.03</v>
@@ -15687,7 +15721,7 @@
     </row>
     <row r="111" ht="15.0" customHeight="1">
       <c r="A111" s="14" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B111" s="16">
         <v>2103.92</v>
@@ -15758,7 +15792,7 @@
     </row>
     <row r="112" ht="15.0" customHeight="1">
       <c r="A112" s="14" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="B112" s="15"/>
       <c r="C112" s="15"/>
@@ -15792,7 +15826,7 @@
       <c r="W112" s="15"/>
     </row>
     <row r="113" ht="15.0" customHeight="1">
-      <c r="A113" s="14" t="s">
+      <c r="A113" s="24" t="s">
         <v>278</v>
       </c>
       <c r="B113" s="15"/>
@@ -15850,7 +15884,7 @@
     </row>
     <row r="114" ht="15.0" customHeight="1">
       <c r="A114" s="14" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B114" s="15"/>
       <c r="C114" s="15"/>
@@ -15895,7 +15929,7 @@
     </row>
     <row r="115" ht="15.0" customHeight="1">
       <c r="A115" s="14" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B115" s="15"/>
       <c r="C115" s="15"/>
@@ -15928,7 +15962,7 @@
     </row>
     <row r="116" ht="15.0" customHeight="1">
       <c r="A116" s="14" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B116" s="15"/>
       <c r="C116" s="15"/>
@@ -15957,7 +15991,7 @@
     </row>
     <row r="117" ht="15.0" customHeight="1">
       <c r="A117" s="14" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="B117" s="15"/>
       <c r="C117" s="15"/>
@@ -15986,7 +16020,7 @@
     </row>
     <row r="118" ht="15.0" customHeight="1">
       <c r="A118" s="17" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B118" s="18">
         <v>142987.55</v>
@@ -16057,7 +16091,7 @@
     </row>
     <row r="119" ht="15.0" customHeight="1">
       <c r="A119" s="17" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B119" s="18">
         <v>273166.49</v>
@@ -16128,7 +16162,7 @@
     </row>
     <row r="120" ht="15.0" customHeight="1">
       <c r="A120" s="14" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B120" s="16">
         <v>379.65</v>
@@ -16199,7 +16233,7 @@
     </row>
     <row r="121" ht="15.0" customHeight="1">
       <c r="A121" s="14" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="B121" s="23">
         <v>-8531.16</v>
@@ -16242,7 +16276,7 @@
     </row>
     <row r="122" ht="15.0" customHeight="1">
       <c r="A122" s="14" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B122" s="22">
         <v>-6.33</v>
@@ -16291,7 +16325,7 @@
     </row>
     <row r="123" ht="15.0" customHeight="1">
       <c r="A123" s="14" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="B123" s="21">
         <v>6.33</v>
@@ -16356,7 +16390,7 @@
     </row>
     <row r="124" ht="15.0" customHeight="1">
       <c r="A124" s="14" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B124" s="23">
         <v>-8531.16</v>
@@ -16421,7 +16455,7 @@
     </row>
     <row r="125" ht="15.0" customHeight="1">
       <c r="A125" s="14" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B125" s="15"/>
       <c r="C125" s="15"/>
@@ -16466,7 +16500,7 @@
     </row>
     <row r="126" ht="15.0" customHeight="1">
       <c r="A126" s="14" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B126" s="15"/>
       <c r="C126" s="15"/>
@@ -16499,7 +16533,7 @@
     </row>
     <row r="127" ht="15.0" customHeight="1">
       <c r="A127" s="14" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B127" s="15">
         <v>193888.21</v>
@@ -16568,7 +16602,7 @@
     </row>
     <row r="128" ht="15.0" customHeight="1">
       <c r="A128" s="14" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B128" s="15"/>
       <c r="C128" s="15"/>
@@ -16611,7 +16645,7 @@
     </row>
     <row r="129" ht="15.0" customHeight="1">
       <c r="A129" s="14" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="B129" s="15"/>
       <c r="C129" s="15"/>
@@ -16640,7 +16674,7 @@
     </row>
     <row r="130" ht="15.0" customHeight="1">
       <c r="A130" s="17" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B130" s="18">
         <v>185736.7</v>
@@ -16782,7 +16816,7 @@
     </row>
     <row r="132" ht="15.0" customHeight="1">
       <c r="A132" s="17" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B132" s="25">
         <v>436.6</v>
@@ -16853,7 +16887,7 @@
     </row>
     <row r="133" ht="15.0" customHeight="1">
       <c r="A133" s="17" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B133" s="18">
         <v>186173.3</v>
@@ -16924,7 +16958,7 @@
     </row>
     <row r="134" ht="15.0" customHeight="1">
       <c r="A134" s="17" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B134" s="18">
         <v>459339.79</v>
@@ -16995,7 +17029,7 @@
     </row>
     <row r="135" ht="15.0" customHeight="1">
       <c r="A135" s="14" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B135" s="16">
         <v>236.74</v>
@@ -17066,7 +17100,7 @@
     </row>
     <row r="136" ht="15.0" customHeight="1">
       <c r="A136" s="14" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B136" s="21">
         <v>3.7</v>
@@ -17137,7 +17171,7 @@
     </row>
     <row r="137" ht="15.0" customHeight="1">
       <c r="A137" s="14" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B137" s="16">
         <v>240.44</v>
@@ -17208,7 +17242,7 @@
     </row>
     <row r="138" ht="15.0" customHeight="1">
       <c r="A138" s="14" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="B138" s="15"/>
       <c r="C138" s="15"/>
@@ -17253,7 +17287,7 @@
     </row>
     <row r="139" ht="15.0" customHeight="1">
       <c r="A139" s="14" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B139" s="15"/>
       <c r="C139" s="15"/>
@@ -17284,7 +17318,7 @@
     </row>
     <row r="140" ht="15.0" customHeight="1">
       <c r="A140" s="14" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="B140" s="15"/>
       <c r="C140" s="15"/>
@@ -17327,7 +17361,7 @@
     </row>
     <row r="141" ht="15.0" customHeight="1">
       <c r="A141" s="14" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B141" s="15"/>
       <c r="C141" s="15"/>
@@ -17356,7 +17390,7 @@
     </row>
     <row r="142" ht="15.0" customHeight="1">
       <c r="A142" s="14" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B142" s="15">
         <v>51777.03</v>
@@ -17401,7 +17435,7 @@
     </row>
     <row r="143" ht="15.0" customHeight="1">
       <c r="A143" s="14" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B143" s="15">
         <v>32768.97</v>
@@ -17432,7 +17466,7 @@
     </row>
     <row r="144" ht="15.0" customHeight="1">
       <c r="A144" s="14" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="B144" s="16">
         <v>5995.38</v>
@@ -17481,7 +17515,7 @@
     </row>
     <row r="145" ht="15.0" customHeight="1">
       <c r="A145" s="14" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="B145" s="15"/>
       <c r="C145" s="15"/>
@@ -17530,7 +17564,7 @@
     </row>
     <row r="146" ht="15.0" customHeight="1">
       <c r="A146" s="14" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B146" s="15"/>
       <c r="C146" s="15"/>
@@ -17569,7 +17603,7 @@
     </row>
     <row r="147" ht="15.0" customHeight="1">
       <c r="A147" s="14" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B147" s="15"/>
       <c r="C147" s="15"/>
@@ -17608,7 +17642,7 @@
     </row>
     <row r="148" ht="15.0" customHeight="1">
       <c r="A148" s="14" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B148" s="15"/>
       <c r="C148" s="15"/>
@@ -17637,7 +17671,7 @@
     </row>
     <row r="149" ht="15.0" customHeight="1">
       <c r="A149" s="14" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B149" s="15">
         <v>13237.3</v>
@@ -17690,7 +17724,7 @@
     </row>
     <row r="150" ht="15.0" customHeight="1">
       <c r="A150" s="14" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="B150" s="15">
         <v>31130.12</v>
@@ -17743,7 +17777,7 @@
     </row>
     <row r="151" ht="15.0" customHeight="1">
       <c r="A151" s="14" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B151" s="15">
         <v>11968.62</v>
@@ -17774,7 +17808,7 @@
     </row>
     <row r="152" ht="15.0" customHeight="1">
       <c r="A152" s="14" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="B152" s="16">
         <v>5517.65</v>
@@ -17819,7 +17853,7 @@
     </row>
     <row r="153" ht="15.0" customHeight="1">
       <c r="A153" s="14" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="B153" s="15">
         <v>11520.95</v>
@@ -17852,7 +17886,7 @@
     </row>
     <row r="154" ht="15.0" customHeight="1">
       <c r="A154" s="14" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="B154" s="16">
         <v>236.74</v>
@@ -17923,7 +17957,7 @@
     </row>
     <row r="155" ht="15.0" customHeight="1">
       <c r="A155" s="14" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="B155" s="21">
         <v>3.7</v>
@@ -17994,7 +18028,7 @@
     </row>
     <row r="156" ht="15.0" customHeight="1">
       <c r="A156" s="14" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="B156" s="16">
         <v>240.44</v>
@@ -18065,7 +18099,7 @@
     </row>
     <row r="157" ht="15.0" customHeight="1">
       <c r="A157" s="14" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B157" s="21">
         <v>1.0</v>
@@ -18998,7 +19032,7 @@
   <sheetData>
     <row r="1" ht="15.0" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -19384,70 +19418,70 @@
         <v>44</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="F15" s="10" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="G15" s="10" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="H15" s="10" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="J15" s="10" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="K15" s="10" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="L15" s="10" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="M15" s="10" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="N15" s="10" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="O15" s="10" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="P15" s="10" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="Q15" s="10" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="R15" s="10" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="S15" s="10" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="T15" s="10" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="U15" s="10" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="V15" s="10" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="W15" s="10" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
     </row>
     <row r="16" ht="15.0" customHeight="1" outlineLevel="1">
@@ -19523,7 +19557,7 @@
     </row>
     <row r="18">
       <c r="A18" s="12" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B18" s="6"/>
       <c r="C18" s="6"/>
@@ -19621,7 +19655,7 @@
     </row>
     <row r="20" ht="15.0" customHeight="1">
       <c r="A20" s="14" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B20" s="15">
         <v>44295.59</v>
@@ -19692,7 +19726,7 @@
     </row>
     <row r="21" ht="15.0" customHeight="1">
       <c r="A21" s="14" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B21" s="16">
         <v>563.03</v>
@@ -19763,7 +19797,7 @@
     </row>
     <row r="22" ht="15.0" customHeight="1">
       <c r="A22" s="14" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B22" s="23">
         <v>-4160.75</v>
@@ -19834,7 +19868,7 @@
     </row>
     <row r="23" ht="15.0" customHeight="1">
       <c r="A23" s="14" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="B23" s="16">
         <v>7887.07</v>
@@ -19905,7 +19939,7 @@
     </row>
     <row r="24" ht="15.0" customHeight="1">
       <c r="A24" s="14" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="B24" s="23">
         <v>-4493.23</v>
@@ -19970,7 +20004,7 @@
     </row>
     <row r="25" ht="15.0" customHeight="1">
       <c r="A25" s="14" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="B25" s="16">
         <v>1707.9</v>
@@ -20025,7 +20059,7 @@
     </row>
     <row r="26" ht="15.0" customHeight="1">
       <c r="A26" s="14" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B26" s="23">
         <v>-2617.52</v>
@@ -20066,7 +20100,7 @@
     </row>
     <row r="27" ht="15.0" customHeight="1">
       <c r="A27" s="14" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B27" s="23">
         <v>-6100.76</v>
@@ -20137,7 +20171,7 @@
     </row>
     <row r="28" ht="15.0" customHeight="1">
       <c r="A28" s="14" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B28" s="15"/>
       <c r="C28" s="15"/>
@@ -20174,7 +20208,7 @@
     </row>
     <row r="29" ht="15.0" customHeight="1">
       <c r="A29" s="14" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="B29" s="15"/>
       <c r="C29" s="15"/>
@@ -20260,7 +20294,7 @@
     </row>
     <row r="31" ht="15.0" customHeight="1">
       <c r="A31" s="14" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="B31" s="15"/>
       <c r="C31" s="15"/>
@@ -20303,7 +20337,7 @@
     </row>
     <row r="32" ht="15.0" customHeight="1">
       <c r="A32" s="14" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="B32" s="15"/>
       <c r="C32" s="15"/>
@@ -20385,7 +20419,7 @@
     </row>
     <row r="34" ht="15.0" customHeight="1">
       <c r="A34" s="14" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="B34" s="23">
         <v>-3392.27</v>
@@ -20454,7 +20488,7 @@
     </row>
     <row r="35" ht="15.0" customHeight="1">
       <c r="A35" s="14" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="B35" s="15"/>
       <c r="C35" s="15"/>
@@ -20487,7 +20521,7 @@
     </row>
     <row r="36" ht="15.0" customHeight="1">
       <c r="A36" s="14" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B36" s="15"/>
       <c r="C36" s="15"/>
@@ -20522,7 +20556,7 @@
     </row>
     <row r="37" ht="15.0" customHeight="1">
       <c r="A37" s="17" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="B37" s="18">
         <v>33689.05</v>
@@ -20593,7 +20627,7 @@
     </row>
     <row r="38" ht="15.0" customHeight="1">
       <c r="A38" s="14" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B38" s="23">
         <v>-820.23</v>
@@ -20664,7 +20698,7 @@
     </row>
     <row r="39" ht="15.0" customHeight="1">
       <c r="A39" s="14" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B39" s="23">
         <v>-3238.58</v>
@@ -20735,7 +20769,7 @@
     </row>
     <row r="40" ht="15.0" customHeight="1">
       <c r="A40" s="14" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="B40" s="16">
         <v>515.98</v>
@@ -20776,7 +20810,7 @@
     </row>
     <row r="41" ht="15.0" customHeight="1">
       <c r="A41" s="14" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="B41" s="15"/>
       <c r="C41" s="15">
@@ -20845,7 +20879,7 @@
     </row>
     <row r="42" ht="15.0" customHeight="1">
       <c r="A42" s="14" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B42" s="16">
         <v>511.27</v>
@@ -20916,7 +20950,7 @@
     </row>
     <row r="43" ht="15.0" customHeight="1">
       <c r="A43" s="14" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="B43" s="15"/>
       <c r="C43" s="15"/>
@@ -20951,7 +20985,7 @@
     </row>
     <row r="44" ht="15.0" customHeight="1">
       <c r="A44" s="14" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B44" s="15"/>
       <c r="C44" s="15"/>
@@ -21008,7 +21042,7 @@
     </row>
     <row r="45" ht="15.0" customHeight="1">
       <c r="A45" s="14" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="B45" s="15"/>
       <c r="C45" s="15"/>
@@ -21051,7 +21085,7 @@
     </row>
     <row r="46" ht="15.0" customHeight="1">
       <c r="A46" s="14" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B46" s="30">
         <v>-118862.87</v>
@@ -21080,7 +21114,7 @@
     </row>
     <row r="47" ht="15.0" customHeight="1">
       <c r="A47" s="17" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="B47" s="26">
         <v>-121894.43</v>
@@ -21151,7 +21185,7 @@
     </row>
     <row r="48" ht="15.0" customHeight="1">
       <c r="A48" s="14" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="B48" s="15">
         <v>22287.38</v>
@@ -21200,7 +21234,7 @@
     </row>
     <row r="49" ht="15.0" customHeight="1">
       <c r="A49" s="14" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B49" s="30">
         <v>-34104.66</v>
@@ -21263,7 +21297,7 @@
     </row>
     <row r="50" ht="15.0" customHeight="1">
       <c r="A50" s="14" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="B50" s="23">
         <v>-9532.24</v>
@@ -21304,7 +21338,7 @@
     </row>
     <row r="51" ht="15.0" customHeight="1">
       <c r="A51" s="14" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="B51" s="16">
         <v>552.05</v>
@@ -21349,7 +21383,7 @@
     </row>
     <row r="52" ht="15.0" customHeight="1">
       <c r="A52" s="14" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B52" s="15">
         <v>0.0</v>
@@ -21388,7 +21422,7 @@
     </row>
     <row r="53" ht="15.0" customHeight="1">
       <c r="A53" s="14" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="B53" s="23">
         <v>-2639.48</v>
@@ -21459,7 +21493,7 @@
     </row>
     <row r="54" ht="15.0" customHeight="1">
       <c r="A54" s="14" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B54" s="15">
         <v>0.0</v>
@@ -21530,7 +21564,7 @@
     </row>
     <row r="55" ht="15.0" customHeight="1">
       <c r="A55" s="14" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="B55" s="16">
         <v>3262.1</v>
@@ -21587,7 +21621,7 @@
     </row>
     <row r="56" ht="15.0" customHeight="1">
       <c r="A56" s="14" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B56" s="23">
         <v>-930.01</v>
@@ -21650,7 +21684,7 @@
     </row>
     <row r="57" ht="15.0" customHeight="1">
       <c r="A57" s="14" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="B57" s="15"/>
       <c r="C57" s="15"/>
@@ -21681,7 +21715,7 @@
     </row>
     <row r="58" ht="15.0" customHeight="1">
       <c r="A58" s="14" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="B58" s="15"/>
       <c r="C58" s="15"/>
@@ -21730,7 +21764,7 @@
     </row>
     <row r="59" ht="15.0" customHeight="1">
       <c r="A59" s="14" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="B59" s="15"/>
       <c r="C59" s="15"/>
@@ -21779,7 +21813,7 @@
     </row>
     <row r="60" ht="15.0" customHeight="1">
       <c r="A60" s="14" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B60" s="15"/>
       <c r="C60" s="15"/>
@@ -21820,7 +21854,7 @@
     </row>
     <row r="61" ht="15.0" customHeight="1">
       <c r="A61" s="14" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="B61" s="15"/>
       <c r="C61" s="15"/>
@@ -21855,7 +21889,7 @@
     </row>
     <row r="62" ht="15.0" customHeight="1">
       <c r="A62" s="17" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="B62" s="26">
         <v>-21104.86</v>
@@ -21926,7 +21960,7 @@
     </row>
     <row r="63" ht="15.0" customHeight="1">
       <c r="A63" s="14" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="B63" s="15">
         <v>132208.51</v>
@@ -21997,7 +22031,7 @@
     </row>
     <row r="64" ht="15.0" customHeight="1">
       <c r="A64" s="14" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="B64" s="30">
         <v>-109310.24</v>
@@ -22050,7 +22084,7 @@
     </row>
     <row r="65" ht="15.0" customHeight="1">
       <c r="A65" s="14" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="B65" s="23">
         <v>-1094.69</v>
@@ -22121,7 +22155,7 @@
     </row>
     <row r="66" ht="15.0" customHeight="1">
       <c r="A66" s="14" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="B66" s="15">
         <v>20847.8</v>
@@ -22192,7 +22226,7 @@
     </row>
     <row r="67" ht="15.0" customHeight="1">
       <c r="A67" s="17" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="B67" s="26">
         <v>-110404.92</v>
@@ -22263,7 +22297,7 @@
     </row>
     <row r="68" ht="15.0" customHeight="1">
       <c r="A68" s="14" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="B68" s="15">
         <v>25618.48</v>
@@ -23257,7 +23291,7 @@
   <sheetData>
     <row r="1" ht="15.0" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -23437,36 +23471,36 @@
         <v>39</v>
       </c>
       <c r="X11" s="7" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="Y11" s="7" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="Z11" s="31" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="AA11" s="32"/>
       <c r="AB11" s="33"/>
       <c r="AC11" s="7" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="AD11" s="7" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="AE11" s="7" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="AF11" s="7" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="AG11" s="7" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="AH11" s="7" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="AI11" s="7" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
     </row>
     <row r="12" ht="15.0" customHeight="1" outlineLevel="1">
@@ -24006,7 +24040,7 @@
     </row>
     <row r="18">
       <c r="A18" s="12" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="B18" s="6"/>
       <c r="C18" s="6"/>
@@ -24114,45 +24148,45 @@
         <v>71</v>
       </c>
       <c r="X19" s="13" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="Y19" s="13" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="Z19" s="13" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="AA19" s="13" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="AB19" s="13" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="AC19" s="13" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="AD19" s="13" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="AE19" s="13" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="AF19" s="13" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="AG19" s="13" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="AH19" s="13" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="AI19" s="13" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
     </row>
     <row r="20" ht="15.0" customHeight="1">
       <c r="A20" s="34" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="B20" s="35"/>
       <c r="C20" s="35"/>
@@ -24191,7 +24225,7 @@
     </row>
     <row r="21" ht="15.0" customHeight="1">
       <c r="A21" s="36" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="B21" s="37">
         <v>748790.16</v>
@@ -24294,7 +24328,7 @@
     </row>
     <row r="22" ht="15.0" customHeight="1">
       <c r="A22" s="36" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="B22" s="37">
         <v>569001.73</v>
@@ -24381,7 +24415,7 @@
     </row>
     <row r="23" ht="15.0" customHeight="1">
       <c r="A23" s="34" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="B23" s="35"/>
       <c r="C23" s="35"/>
@@ -24420,7 +24454,7 @@
     </row>
     <row r="24" ht="15.0" customHeight="1">
       <c r="A24" s="36" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="B24" s="37">
         <v>614278.41</v>
@@ -24523,7 +24557,7 @@
     </row>
     <row r="25" ht="15.0" customHeight="1">
       <c r="A25" s="36" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B25" s="37">
         <v>513266.8</v>
@@ -24610,7 +24644,7 @@
     </row>
     <row r="26" ht="15.0" customHeight="1">
       <c r="A26" s="34" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="B26" s="35"/>
       <c r="C26" s="35"/>
@@ -24649,7 +24683,7 @@
     </row>
     <row r="27" ht="15.0" customHeight="1">
       <c r="A27" s="36" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B27" s="38">
         <v>2554.76</v>
@@ -24754,7 +24788,7 @@
     </row>
     <row r="28" ht="15.0" customHeight="1">
       <c r="A28" s="36" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="B28" s="38">
         <v>2199.94</v>
@@ -24851,7 +24885,7 @@
     </row>
     <row r="29" ht="15.0" customHeight="1">
       <c r="A29" s="34" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="B29" s="35"/>
       <c r="C29" s="35"/>
@@ -24890,7 +24924,7 @@
     </row>
     <row r="30" ht="15.0" customHeight="1">
       <c r="A30" s="36" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="B30" s="41">
         <v>4.96</v>
@@ -24991,7 +25025,7 @@
     </row>
     <row r="31" ht="15.0" customHeight="1">
       <c r="A31" s="36" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="B31" s="41">
         <v>4.94</v>
@@ -25076,7 +25110,7 @@
     </row>
     <row r="32" ht="15.0" customHeight="1">
       <c r="A32" s="34" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="B32" s="35"/>
       <c r="C32" s="35"/>
@@ -25115,7 +25149,7 @@
     </row>
     <row r="33" ht="15.0" customHeight="1">
       <c r="A33" s="36" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="B33" s="41">
         <v>0.43</v>
@@ -25216,7 +25250,7 @@
     </row>
     <row r="34" ht="15.0" customHeight="1">
       <c r="A34" s="36" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="B34" s="41">
         <v>0.43</v>
@@ -25301,7 +25335,7 @@
     </row>
     <row r="35" ht="15.0" customHeight="1">
       <c r="A35" s="36" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="B35" s="41">
         <v>0.43</v>
@@ -25406,7 +25440,7 @@
     </row>
     <row r="36" ht="15.0" customHeight="1">
       <c r="A36" s="36" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="B36" s="41">
         <v>0.43</v>
@@ -25503,7 +25537,7 @@
     </row>
     <row r="37" ht="15.0" customHeight="1">
       <c r="A37" s="34" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B37" s="35"/>
       <c r="C37" s="35"/>
@@ -25542,7 +25576,7 @@
     </row>
     <row r="38" ht="15.0" customHeight="1">
       <c r="A38" s="36" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="B38" s="40">
         <v>3.26</v>
@@ -25629,7 +25663,7 @@
     </row>
     <row r="39" ht="15.0" customHeight="1">
       <c r="A39" s="36" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="B39" s="40">
         <v>3.55</v>
@@ -25708,7 +25742,7 @@
     </row>
     <row r="40" ht="15.0" customHeight="1">
       <c r="A40" s="34" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="B40" s="35"/>
       <c r="C40" s="35"/>
@@ -25747,7 +25781,7 @@
     </row>
     <row r="41" ht="15.0" customHeight="1">
       <c r="A41" s="36" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="B41" s="37"/>
       <c r="C41" s="40">
@@ -25812,7 +25846,7 @@
     </row>
     <row r="42" ht="15.0" customHeight="1">
       <c r="A42" s="36" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="B42" s="37"/>
       <c r="C42" s="40">
@@ -25863,7 +25897,7 @@
     </row>
     <row r="43" ht="15.0" customHeight="1">
       <c r="A43" s="34" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="B43" s="35"/>
       <c r="C43" s="35"/>
@@ -25902,7 +25936,7 @@
     </row>
     <row r="44" ht="15.0" customHeight="1">
       <c r="A44" s="36" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="B44" s="40">
         <v>1.54</v>
@@ -26009,7 +26043,7 @@
     </row>
     <row r="45" ht="15.0" customHeight="1">
       <c r="A45" s="36" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="B45" s="40">
         <v>1.6</v>
@@ -26108,7 +26142,7 @@
     </row>
     <row r="46" ht="15.0" customHeight="1">
       <c r="A46" s="34" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="B46" s="35"/>
       <c r="C46" s="35"/>
@@ -26147,7 +26181,7 @@
     </row>
     <row r="47" ht="15.0" customHeight="1">
       <c r="A47" s="36" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="B47" s="40">
         <v>20.16</v>
@@ -26246,7 +26280,7 @@
     </row>
     <row r="48" ht="15.0" customHeight="1">
       <c r="A48" s="36" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="B48" s="40">
         <v>20.26</v>
@@ -26331,7 +26365,7 @@
     </row>
     <row r="49" ht="15.0" customHeight="1">
       <c r="A49" s="34" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="B49" s="35"/>
       <c r="C49" s="35"/>
@@ -26370,7 +26404,7 @@
     </row>
     <row r="50" ht="15.0" customHeight="1">
       <c r="A50" s="36" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="B50" s="40">
         <v>22.22</v>
@@ -26477,7 +26511,7 @@
     </row>
     <row r="51" ht="15.0" customHeight="1">
       <c r="A51" s="36" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="B51" s="40">
         <v>17.64</v>
@@ -26576,7 +26610,7 @@
     </row>
     <row r="52" ht="15.0" customHeight="1">
       <c r="A52" s="34" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="B52" s="35"/>
       <c r="C52" s="35"/>
@@ -26615,7 +26649,7 @@
     </row>
     <row r="53" ht="15.0" customHeight="1">
       <c r="A53" s="36" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="B53" s="40">
         <v>45.41</v>
@@ -26722,7 +26756,7 @@
     </row>
     <row r="54" ht="15.0" customHeight="1">
       <c r="A54" s="36" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="B54" s="40">
         <v>26.32</v>
@@ -26821,7 +26855,7 @@
     </row>
     <row r="55" ht="15.0" customHeight="1">
       <c r="A55" s="34" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="B55" s="35"/>
       <c r="C55" s="35"/>
@@ -26860,7 +26894,7 @@
     </row>
     <row r="56" ht="15.0" customHeight="1">
       <c r="A56" s="36" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="B56" s="40">
         <v>29.49</v>
@@ -26967,7 +27001,7 @@
     </row>
     <row r="57" ht="15.0" customHeight="1">
       <c r="A57" s="36" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="B57" s="40">
         <v>3.55</v>
@@ -27054,7 +27088,7 @@
     </row>
     <row r="58" ht="15.0" customHeight="1">
       <c r="A58" s="34" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="B58" s="35"/>
       <c r="C58" s="35"/>
@@ -27093,7 +27127,7 @@
     </row>
     <row r="59" ht="15.0" customHeight="1">
       <c r="A59" s="36" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="B59" s="39">
         <v>-1.86</v>
@@ -27198,7 +27232,7 @@
     </row>
     <row r="60" ht="15.0" customHeight="1">
       <c r="A60" s="36" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="B60" s="40">
         <v>1.86</v>
@@ -27295,7 +27329,7 @@
     </row>
     <row r="61" ht="15.0" customHeight="1">
       <c r="A61" s="34" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="B61" s="35"/>
       <c r="C61" s="35"/>
@@ -27334,7 +27368,7 @@
     </row>
     <row r="62" ht="15.0" customHeight="1">
       <c r="A62" s="36" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="B62" s="40">
         <v>1.91</v>
@@ -27437,7 +27471,7 @@
     </row>
     <row r="63" ht="15.0" customHeight="1">
       <c r="A63" s="36" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="B63" s="40">
         <v>1.83</v>
@@ -27524,7 +27558,7 @@
     </row>
     <row r="64" ht="15.0" customHeight="1">
       <c r="A64" s="34" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="B64" s="35"/>
       <c r="C64" s="35"/>
@@ -27563,7 +27597,7 @@
     </row>
     <row r="65" ht="15.0" customHeight="1">
       <c r="A65" s="36" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="B65" s="40">
         <v>16.76</v>
@@ -27666,7 +27700,7 @@
     </row>
     <row r="66" ht="15.0" customHeight="1">
       <c r="A66" s="36" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="B66" s="40">
         <v>14.53</v>
@@ -27753,7 +27787,7 @@
     </row>
     <row r="67" ht="15.0" customHeight="1">
       <c r="A67" s="34" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="B67" s="35"/>
       <c r="C67" s="35"/>
@@ -27792,7 +27826,7 @@
     </row>
     <row r="68" ht="15.0" customHeight="1">
       <c r="A68" s="36" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="B68" s="40">
         <v>22.04</v>
@@ -27893,7 +27927,7 @@
     </row>
     <row r="69" ht="15.0" customHeight="1">
       <c r="A69" s="36" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="B69" s="40">
         <v>20.29</v>
@@ -27978,7 +28012,7 @@
     </row>
     <row r="70" ht="15.0" customHeight="1">
       <c r="A70" s="34" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="B70" s="35"/>
       <c r="C70" s="35"/>
@@ -28017,7 +28051,7 @@
     </row>
     <row r="71" ht="15.0" customHeight="1">
       <c r="A71" s="36" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="B71" s="40">
         <v>25.05</v>
@@ -28116,7 +28150,7 @@
     </row>
     <row r="72" ht="15.0" customHeight="1">
       <c r="A72" s="36" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="B72" s="40">
         <v>23.07</v>

</xml_diff>